<commit_message>
Add notes, throughput and unit-labelled latency columns to results.xlsx
Matches the required columns in GUIDE section 6.1 (Training: notes;
Inference: images/s; Latency: units in column names).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submissions/2A202602437_vu_duc_thien/results.xlsx
+++ b/submissions/2A202602437_vu_duc_thien/results.xlsx
@@ -942,7 +942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O18"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -960,6 +960,7 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="27" customWidth="1" min="14" max="14"/>
     <col width="23" customWidth="1" min="15" max="15"/>
+    <col width="48" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1045,6 +1046,11 @@
           <t>GPU</t>
         </is>
       </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>ghi chú</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1104,6 +1110,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>mốc; 3 seed để đo nhiễu</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1163,6 +1174,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>mốc; 3 seed để đo nhiễu</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1222,6 +1238,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>mốc; 3 seed để đo nhiễu</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1281,6 +1302,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1340,6 +1366,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1399,6 +1430,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1458,6 +1494,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1517,6 +1558,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1576,6 +1622,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1635,6 +1686,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1694,6 +1750,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1753,6 +1814,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1812,6 +1878,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1871,6 +1942,11 @@
           <t>Tesla T4</t>
         </is>
       </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>1 seed</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1928,6 +2004,11 @@
       <c r="O18" t="inlineStr">
         <is>
           <t>NVIDIA A100-SXM4-40GB</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>1 seed; chạy trên NVIDIA A100-SXM4-40GB (các lần khác trên T4)</t>
         </is>
       </c>
     </row>
@@ -1942,7 +2023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1957,10 +2038,11 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="19" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2033,20 +2115,25 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
+          <t>thông lượng b1 (ảnh/s)</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
           <t>chi phí so với I00 (lần)</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>T (khớp trên val)</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>ECE val trước TS</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>ECE val sau TS (khớp chéo 2 nửa)</t>
         </is>
@@ -2096,11 +2183,14 @@
         <v>12.01379516937778</v>
       </c>
       <c r="M4" s="3" t="n">
+        <v>89.11146556678341</v>
+      </c>
+      <c r="N4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N4" s="3" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
       <c r="P4" s="3" t="inlineStr"/>
+      <c r="Q4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2146,11 +2236,14 @@
         <v>24.34776191014862</v>
       </c>
       <c r="M5" s="3" t="n">
+        <v>44.67271506998996</v>
+      </c>
+      <c r="N5" s="3" t="n">
         <v>1.994762696361081</v>
       </c>
-      <c r="N5" s="3" t="inlineStr"/>
       <c r="O5" s="3" t="inlineStr"/>
       <c r="P5" s="3" t="inlineStr"/>
+      <c r="Q5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2196,11 +2289,14 @@
         <v>24.34776191014862</v>
       </c>
       <c r="M6" s="3" t="n">
+        <v>44.67271506998996</v>
+      </c>
+      <c r="N6" s="3" t="n">
         <v>1.994762696361081</v>
       </c>
-      <c r="N6" s="3" t="inlineStr"/>
       <c r="O6" s="3" t="inlineStr"/>
       <c r="P6" s="3" t="inlineStr"/>
+      <c r="Q6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2246,11 +2342,14 @@
         <v>58.8777633202608</v>
       </c>
       <c r="M7" s="3" t="n">
+        <v>17.82258962986617</v>
+      </c>
+      <c r="N7" s="3" t="n">
         <v>4.999916814414842</v>
       </c>
-      <c r="N7" s="3" t="inlineStr"/>
       <c r="O7" s="3" t="inlineStr"/>
       <c r="P7" s="3" t="inlineStr"/>
+      <c r="Q7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2296,11 +2395,14 @@
         <v>58.8777633202608</v>
       </c>
       <c r="M8" s="3" t="n">
+        <v>17.82258962986617</v>
+      </c>
+      <c r="N8" s="3" t="n">
         <v>4.999916814414842</v>
       </c>
-      <c r="N8" s="3" t="inlineStr"/>
       <c r="O8" s="3" t="inlineStr"/>
       <c r="P8" s="3" t="inlineStr"/>
+      <c r="Q8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2346,11 +2448,14 @@
         <v>126.2826702101484</v>
       </c>
       <c r="M9" s="3" t="n">
+        <v>9.015728528906529</v>
+      </c>
+      <c r="N9" s="3" t="n">
         <v>9.884000530968882</v>
       </c>
-      <c r="N9" s="3" t="inlineStr"/>
       <c r="O9" s="3" t="inlineStr"/>
       <c r="P9" s="3" t="inlineStr"/>
+      <c r="Q9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2396,11 +2501,14 @@
         <v>126.2826702101484</v>
       </c>
       <c r="M10" s="3" t="n">
+        <v>9.015728528906529</v>
+      </c>
+      <c r="N10" s="3" t="n">
         <v>9.884000530968882</v>
       </c>
-      <c r="N10" s="3" t="inlineStr"/>
       <c r="O10" s="3" t="inlineStr"/>
       <c r="P10" s="3" t="inlineStr"/>
+      <c r="Q10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -2446,11 +2554,14 @@
         <v>39.63201569002195</v>
       </c>
       <c r="M11" s="5" t="n">
+        <v>30.38097868765697</v>
+      </c>
+      <c r="N11" s="5" t="n">
         <v>2.933133474169058</v>
       </c>
-      <c r="N11" s="5" t="inlineStr"/>
       <c r="O11" s="5" t="inlineStr"/>
       <c r="P11" s="5" t="inlineStr"/>
+      <c r="Q11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2496,11 +2607,14 @@
         <v>25.52180390057403</v>
       </c>
       <c r="M12" s="3" t="n">
+        <v>43.74579015220772</v>
+      </c>
+      <c r="N12" s="3" t="n">
         <v>2.037029512022341</v>
       </c>
-      <c r="N12" s="3" t="inlineStr"/>
       <c r="O12" s="3" t="inlineStr"/>
       <c r="P12" s="3" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2546,11 +2660,14 @@
         <v>11.89911860989014</v>
       </c>
       <c r="M13" s="3" t="n">
+        <v>90.50827501107659</v>
+      </c>
+      <c r="N13" s="3" t="n">
         <v>0.9845670526355494</v>
       </c>
-      <c r="N13" s="3" t="inlineStr"/>
       <c r="O13" s="3" t="inlineStr"/>
       <c r="P13" s="3" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2596,11 +2713,14 @@
         <v>12.86162427977616</v>
       </c>
       <c r="M14" s="3" t="n">
+        <v>89.05435583586068</v>
+      </c>
+      <c r="N14" s="3" t="n">
         <v>1.000641290708205</v>
       </c>
-      <c r="N14" s="3" t="inlineStr"/>
       <c r="O14" s="3" t="inlineStr"/>
       <c r="P14" s="3" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2646,15 +2766,18 @@
         <v>12.68663648937945</v>
       </c>
       <c r="M15" s="3" t="n">
+        <v>90.22573757565128</v>
+      </c>
+      <c r="N15" s="3" t="n">
         <v>0.9876501756726171</v>
       </c>
-      <c r="N15" s="3" t="n">
+      <c r="O15" s="3" t="n">
         <v>1.27628860265234</v>
       </c>
-      <c r="O15" s="3" t="n">
+      <c r="P15" s="3" t="n">
         <v>0.0090579123013064</v>
       </c>
-      <c r="P15" s="3" t="n">
+      <c r="Q15" s="3" t="n">
         <v>0.008914796014019601</v>
       </c>
     </row>
@@ -2702,11 +2825,14 @@
         <v>15.45504605050155</v>
       </c>
       <c r="M16" s="3" t="n">
+        <v>86.19540878551578</v>
+      </c>
+      <c r="N16" s="3" t="n">
         <v>1.033830766886016</v>
       </c>
-      <c r="N16" s="3" t="inlineStr"/>
       <c r="O16" s="3" t="inlineStr"/>
       <c r="P16" s="3" t="inlineStr"/>
+      <c r="Q16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2752,11 +2878,14 @@
         <v>13.8898818898997</v>
       </c>
       <c r="M17" s="3" t="n">
+        <v>89.87137473981711</v>
+      </c>
+      <c r="N17" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N17" s="3" t="inlineStr"/>
       <c r="O17" s="3" t="inlineStr"/>
       <c r="P17" s="3" t="inlineStr"/>
+      <c r="Q17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2802,11 +2931,14 @@
         <v>27.09850498002652</v>
       </c>
       <c r="M18" s="3" t="n">
+        <v>46.0883110569787</v>
+      </c>
+      <c r="N18" s="3" t="n">
         <v>1.94998195157791</v>
       </c>
-      <c r="N18" s="3" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr"/>
       <c r="P18" s="3" t="inlineStr"/>
+      <c r="Q18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2852,11 +2984,14 @@
         <v>27.09850498002652</v>
       </c>
       <c r="M19" s="3" t="n">
+        <v>46.0883110569787</v>
+      </c>
+      <c r="N19" s="3" t="n">
         <v>1.94998195157791</v>
       </c>
-      <c r="N19" s="3" t="inlineStr"/>
       <c r="O19" s="3" t="inlineStr"/>
       <c r="P19" s="3" t="inlineStr"/>
+      <c r="Q19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2902,11 +3037,14 @@
         <v>58.42512614967746</v>
       </c>
       <c r="M20" s="3" t="n">
+        <v>18.51427137901007</v>
+      </c>
+      <c r="N20" s="3" t="n">
         <v>4.854167517588932</v>
       </c>
-      <c r="N20" s="3" t="inlineStr"/>
       <c r="O20" s="3" t="inlineStr"/>
       <c r="P20" s="3" t="inlineStr"/>
+      <c r="Q20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2952,11 +3090,14 @@
         <v>58.42512614967746</v>
       </c>
       <c r="M21" s="3" t="n">
+        <v>18.51427137901007</v>
+      </c>
+      <c r="N21" s="3" t="n">
         <v>4.854167517588932</v>
       </c>
-      <c r="N21" s="3" t="inlineStr"/>
       <c r="O21" s="3" t="inlineStr"/>
       <c r="P21" s="3" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3002,11 +3143,14 @@
         <v>114.9548796402451</v>
       </c>
       <c r="M22" s="3" t="n">
+        <v>9.166778642699466</v>
+      </c>
+      <c r="N22" s="3" t="n">
         <v>9.804030209826411</v>
       </c>
-      <c r="N22" s="3" t="inlineStr"/>
       <c r="O22" s="3" t="inlineStr"/>
       <c r="P22" s="3" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3052,11 +3196,14 @@
         <v>114.9548796402451</v>
       </c>
       <c r="M23" s="3" t="n">
+        <v>9.166778642699466</v>
+      </c>
+      <c r="N23" s="3" t="n">
         <v>9.804030209826411</v>
       </c>
-      <c r="N23" s="3" t="inlineStr"/>
       <c r="O23" s="3" t="inlineStr"/>
       <c r="P23" s="3" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3102,15 +3249,18 @@
         <v>13.51364008976816</v>
       </c>
       <c r="M24" s="3" t="n">
+        <v>91.51813996938895</v>
+      </c>
+      <c r="N24" s="3" t="n">
         <v>0.9820061330997042</v>
       </c>
-      <c r="N24" s="3" t="n">
+      <c r="O24" s="3" t="n">
         <v>0.621857248701803</v>
       </c>
-      <c r="O24" s="3" t="n">
+      <c r="P24" s="3" t="n">
         <v>0.09175426691463071</v>
       </c>
-      <c r="P24" s="3" t="n">
+      <c r="Q24" s="3" t="n">
         <v>0.011136918306741</v>
       </c>
     </row>
@@ -3158,11 +3308,14 @@
         <v>14.18355735973819</v>
       </c>
       <c r="M25" s="3" t="n">
+        <v>87.64757715664472</v>
+      </c>
+      <c r="N25" s="3" t="n">
         <v>1.025372037143685</v>
       </c>
-      <c r="N25" s="3" t="inlineStr"/>
       <c r="O25" s="3" t="inlineStr"/>
       <c r="P25" s="3" t="inlineStr"/>
+      <c r="Q25" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4115,18 +4268,18 @@
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4139,12 +4292,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>config</t>
+          <t>cấu hình</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>gpu</t>
+          <t>GPU</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -4159,52 +4312,52 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>img_size</t>
+          <t>độ phân giải</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>fused_bn</t>
+          <t>gộp BN</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>k_views</t>
+          <t>K (view)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>p50</t>
+          <t>p50 (ms)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>p95</t>
+          <t>p95 (ms)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>p99</t>
+          <t>p99 (ms)</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>trung bình (ms)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>images_per_s</t>
+          <t>thông lượng (ảnh/s)</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>n_iters</t>
+          <t>số lần đo</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>warmup</t>
+          <t>warmup (lần)</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -4214,7 +4367,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>preprocessing</t>
+          <t>tiền xử lý</t>
         </is>
       </c>
     </row>

</xml_diff>